<commit_message>
Subir el margen al 50 % en las cotizaciones internas y en la de Tyler
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0137o8WSxNvVuvENWjtHj8Xx
</commit_message>
<xml_diff>
--- a/cotizaciones/Estimate_Yellowstone_Club_Stone_Floor.xlsx
+++ b/cotizaciones/Estimate_Yellowstone_Club_Stone_Floor.xlsx
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>7915</v>
+        <v>10290</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>6375</v>
+        <v>8285</v>
       </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="D23" s="16" t="n">
-        <v>6820</v>
+        <v>8860</v>
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="D24" s="16" t="n">
-        <v>6180</v>
+        <v>8030</v>
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Subir el margen al 55 % en las cotizaciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0137o8WSxNvVuvENWjtHj8Xx
</commit_message>
<xml_diff>
--- a/cotizaciones/Estimate_Yellowstone_Club_Stone_Floor.xlsx
+++ b/cotizaciones/Estimate_Yellowstone_Club_Stone_Floor.xlsx
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>10290</v>
+        <v>11430</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>8285</v>
+        <v>9205</v>
       </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="D23" s="16" t="n">
-        <v>8860</v>
+        <v>9845</v>
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="D24" s="16" t="n">
-        <v>8030</v>
+        <v>8920</v>
       </c>
       <c r="E24" s="17" t="inlineStr">
         <is>

</xml_diff>